<commit_message>
Deconstruct : requirements du workflow Import Mensuel Finance
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mkbwf9F7YipotQMesNF3MR
</commit_message>
<xml_diff>
--- a/outputs/deconstruct-extraction-fichier-finance-suivi.xlsx
+++ b/outputs/deconstruct-extraction-fichier-finance-suivi.xlsx
@@ -403,52 +403,56 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -707,126 +711,126 @@
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -849,194 +853,194 @@
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6" t="s">
+      <c r="C5" s="8"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6" t="s">
+      <c r="D7" s="7"/>
+      <c r="E7" s="7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6" t="s">
+      <c r="C9" s="8"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6" t="s">
+      <c r="C10" s="8"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -1063,142 +1067,142 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="8" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="10" t="s">
+      <c r="A11" s="3"/>
+      <c r="B11" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2" t="str">
+      <c r="C11" s="3"/>
+      <c r="D11" s="3" t="str">
         <f aca="false">COUNTIF(D5:D9,"Terminé")&amp;" / "&amp;COUNTA(A5:A9)</f>
         <v>0 / 5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="10" t="s">
+      <c r="A12" s="3"/>
+      <c r="B12" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="11" t="n">
+      <c r="C12" s="3"/>
+      <c r="D12" s="12" t="n">
         <f aca="false">COUNTIF(D5:D9,"Terminé")/COUNTA(A5:A9)</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Deconstruct : mise à jour de la feuille de suivi (chapitres terminés)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mkbwf9F7YipotQMesNF3MR
</commit_message>
<xml_diff>
--- a/outputs/deconstruct-extraction-fichier-finance-suivi.xlsx
+++ b/outputs/deconstruct-extraction-fichier-finance-suivi.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="78">
   <si>
     <t xml:space="preserve">Extraction mensuelle du fichier finance — Fiche workflow</t>
   </si>
@@ -42,7 +42,7 @@
     <t xml:space="preserve">Workflow</t>
   </si>
   <si>
-    <t xml:space="preserve">Extraction mensuelle du fichier finance</t>
+    <t xml:space="preserve">Import Mensuel Finance (identifiant : import-mensuel-finance)</t>
   </si>
   <si>
     <t xml:space="preserve">Rapport d'opportunités (#1)</t>
@@ -51,7 +51,7 @@
     <t xml:space="preserve">Déclencheur</t>
   </si>
   <si>
-    <t xml:space="preserve">Réception du Google Sheet mensuel de la finance</t>
+    <t xml:space="preserve">Réception du Google Sheet « Xbh Contracts Financial performance : [Mois] [Année] » vers le 15 du mois ; lancement manuel avec le mois</t>
   </si>
   <si>
     <t xml:space="preserve">Entretien Analyze</t>
@@ -60,7 +60,7 @@
     <t xml:space="preserve">Livrable</t>
   </si>
   <si>
-    <t xml:space="preserve">Sheet personnel mis à jour avec les données du mois, lisible par Looker Studio, avec contrôle des totaux</t>
+    <t xml:space="preserve">Database XBH [Mois] [Année] remplie par WBS exact, onglets « À traiter à la main » et « Contrôle »</t>
   </si>
   <si>
     <t xml:space="preserve">Chemin</t>
@@ -96,7 +96,7 @@
     <t xml:space="preserve">Statut</t>
   </si>
   <si>
-    <t xml:space="preserve">Deconstruct en cours — chapitre 1</t>
+    <t xml:space="preserve">Deconstruct terminé — requirements dans outputs/import-mensuel-finance/</t>
   </si>
   <si>
     <t xml:space="preserve">Session du 2026-10-26</t>
@@ -126,6 +126,9 @@
     <t xml:space="preserve">Quel objectif ce workflow soutient-il ? (peut être personnel)</t>
   </si>
   <si>
+    <t xml:space="preserve">Gagner du temps et sécuriser la transmission des données qui alimentent le dashboard HCare du service</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chapitre 1</t>
   </si>
   <si>
@@ -135,6 +138,9 @@
     <t xml:space="preserve">Quand ça marche, qu'est-ce qui change concrètement, et pour qui ?</t>
   </si>
   <si>
+    <t xml:space="preserve">Database du mois constituée rapidement et sans erreur ; dashboard disponible plus tôt pour le service, chiffres garantis conformes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chapitre 1 — question en cours</t>
   </si>
   <si>
@@ -144,7 +150,7 @@
     <t xml:space="preserve">Qu'est-ce qu'on compte ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Temps passé sur le transfert finance → Sheet personnel, par clôture mensuelle</t>
+    <t xml:space="preserve">(1) Temps réception → validation · (2) Contrats oubliés et écarts inexpliqués par clôture</t>
   </si>
   <si>
     <t xml:space="preserve">Baseline</t>
@@ -153,10 +159,10 @@
     <t xml:space="preserve">Quel est le chiffre aujourd'hui ?</t>
   </si>
   <si>
-    <t xml:space="preserve">1 à 2 jours de travail par clôture mensuelle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimé</t>
+    <t xml:space="preserve">(1) 1 à 2 jours par clôture · (2) Inconnue — à mesurer avant mise en service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimé / Inconnue</t>
   </si>
   <si>
     <t xml:space="preserve">Chapitre 1 (donné par Baptiste en Analyze)</t>
@@ -168,6 +174,9 @@
     <t xml:space="preserve">Quel chiffre viser avec le workflow révisé ?</t>
   </si>
   <si>
+    <t xml:space="preserve">(1) Une matinée · (2) 0 contrat oublié, 0 écart inexpliqué</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chapitre 5</t>
   </si>
   <si>
@@ -177,6 +186,9 @@
     <t xml:space="preserve">Combien de temps après la mise en service peut-on lire ce chiffre ?</t>
   </si>
   <si>
+    <t xml:space="preserve">Dès la première clôture suivant la mise en service</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pistes de réponse évoquées pour « Desired Outcome »</t>
   </si>
   <si>
@@ -213,16 +225,13 @@
     <t xml:space="preserve">Objectif, résultat attendu, mesure, situation actuelle</t>
   </si>
   <si>
-    <t xml:space="preserve">En cours</t>
+    <t xml:space="preserve">Terminé</t>
   </si>
   <si>
     <t xml:space="preserve">Périmètre et nom</t>
   </si>
   <si>
     <t xml:space="preserve">Un déclencheur, un livrable ; nom et identifiant du workflow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À faire</t>
   </si>
   <si>
     <t xml:space="preserve">Cartographie des étapes</t>
@@ -408,51 +417,51 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -716,26 +725,26 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -746,7 +755,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
@@ -757,7 +766,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
@@ -768,7 +777,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
@@ -779,7 +788,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
@@ -790,7 +799,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
         <v>16</v>
       </c>
@@ -801,7 +810,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
         <v>18</v>
       </c>
@@ -812,7 +821,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
         <v>21</v>
       </c>
@@ -823,7 +832,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
         <v>23</v>
       </c>
@@ -860,7 +869,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>26</v>
       </c>
@@ -869,7 +878,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>27</v>
       </c>
@@ -878,14 +887,14 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -902,141 +911,149 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="8"/>
+      <c r="C5" s="7" t="s">
+        <v>34</v>
+      </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="8"/>
+        <v>37</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>38</v>
+      </c>
       <c r="D6" s="7"/>
       <c r="E6" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>45</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="8"/>
+        <v>49</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>50</v>
+      </c>
       <c r="D9" s="7"/>
       <c r="E9" s="7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="8"/>
+        <v>53</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>54</v>
+      </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
-        <v>51</v>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -1073,138 +1090,138 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>66</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>69</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>73</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>75</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3"/>
       <c r="B11" s="11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3" t="str">
         <f aca="false">COUNTIF(D5:D9,"Terminé")&amp;" / "&amp;COUNTA(A5:A9)</f>
-        <v>0 / 5</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5 / 5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3"/>
       <c r="B12" s="11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="12" t="n">
         <f aca="false">COUNTIF(D5:D9,"Terminé")/COUNTA(A5:A9)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>